<commit_message>
Se implementa la resolución de nombres de catálogo en el mapeo de datos de empleados, mejorando la carga de información en la plantilla de exportación. Se actualizan los selectores en la vista de edición de empleados para permitir la habilitación y deshabilitación de la edición, y se añaden mensajes de error para los campos del formulario. Además, se ajustan estilos en la interfaz para mejorar la usabilidad.
</commit_message>
<xml_diff>
--- a/storage/templates/plantilla-masivos.xlsx
+++ b/storage/templates/plantilla-masivos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manuel.espinosa\Desktop\GH DOCS CONTRATACION\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SJSEGURIDAD\storage\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F094314A-B0E1-40D6-B86C-CBCF8E155BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{170707BF-FB26-491E-AA7B-B69611AE30E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="718" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="EMPLEADOS" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EMPLEADOS!$A$2:$BJ$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">EMPLEADOS!$A$2:$BJ$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t>TMPCEDULA.C15</t>
   </si>
@@ -514,143 +514,12 @@
 SI-1
 NO-0</t>
   </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>230301</t>
-  </si>
-  <si>
-    <t>PORVENIR</t>
-  </si>
-  <si>
-    <t>N5</t>
-  </si>
-  <si>
-    <t>01</t>
-  </si>
-  <si>
-    <t>SALARIO LEY 100</t>
-  </si>
-  <si>
-    <t>230201</t>
-  </si>
-  <si>
-    <t>PROTECCION</t>
-  </si>
-  <si>
-    <t>002</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>BANCOLOMBIA</t>
-  </si>
-  <si>
-    <t>AGUILAR MARTHEY JOSE ORLANDO</t>
-  </si>
-  <si>
-    <t>AGUILAR</t>
-  </si>
-  <si>
-    <t>MARTHEY</t>
-  </si>
-  <si>
-    <t>JOSE</t>
-  </si>
-  <si>
-    <t>ORLANDO</t>
-  </si>
-  <si>
-    <t>CL 3 5 40</t>
-  </si>
-  <si>
-    <t>joseorlandoaguilarmarthey@gmail.com</t>
-  </si>
-  <si>
-    <t>54001</t>
-  </si>
-  <si>
-    <t>CUCUTA</t>
-  </si>
-  <si>
-    <t>007</t>
-  </si>
-  <si>
-    <t>ESCOLTA</t>
-  </si>
-  <si>
-    <t>1007</t>
-  </si>
-  <si>
-    <t>76978582601</t>
-  </si>
-  <si>
-    <t>0405</t>
-  </si>
-  <si>
-    <t>UNION TEMPORAL NCCTS 2026</t>
-  </si>
-  <si>
-    <t>EPS005</t>
-  </si>
-  <si>
-    <t>SANITAS</t>
-  </si>
-  <si>
-    <t>ARL AXA COLPATRIA</t>
-  </si>
-  <si>
-    <t>CCF37</t>
-  </si>
-  <si>
-    <t>COMFANORTE- CAJA DE COMPENSACI</t>
-  </si>
-  <si>
-    <t>88196928</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>OBRA LABOR</t>
-  </si>
-  <si>
-    <t>OCCIDENTE</t>
-  </si>
-  <si>
-    <t>L003</t>
-  </si>
-  <si>
-    <t>ESCOLTAS</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>CLIENTE EXTERNO</t>
-  </si>
-  <si>
-    <t>ACTIVIDADES DE SEGURIDAD PRIVADA, INCLUYE SERVICIOS DE GUARDIAS DE SEGURIDAD.</t>
-  </si>
-  <si>
-    <t>3108921091</t>
-  </si>
-  <si>
-    <t>14-04</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="3">
-    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="165" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-  </numFmts>
-  <fonts count="11">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -673,14 +542,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -697,36 +558,8 @@
       <sz val="9"/>
       <name val="Times New Roman"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="8"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -736,12 +569,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -770,15 +597,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -816,71 +641,15 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="6">
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
-    <cellStyle name="Moneda" xfId="5" builtinId="4"/>
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
-    <cellStyle name="Normal 2 3" xfId="3" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
-    <cellStyle name="Normal 3" xfId="4" xr:uid="{D51D5584-9622-4DB0-9554-03F0E241CF90}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
+    <cellStyle name="Normal 2 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
+    <cellStyle name="Normal 3" xfId="3" xr:uid="{D51D5584-9622-4DB0-9554-03F0E241CF90}"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1199,7 +968,7 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:BJ3"/>
+  <dimension ref="A1:BJ2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -1535,7 +1304,7 @@
       <c r="AA2" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="AB2" s="27" t="s">
+      <c r="AB2" s="13" t="s">
         <v>89</v>
       </c>
       <c r="AC2" s="8" t="s">
@@ -1639,186 +1408,6 @@
       </c>
       <c r="BJ2" s="8" t="s">
         <v>123</v>
-      </c>
-    </row>
-    <row r="3" spans="1:62" s="15" customFormat="1" ht="12.6" customHeight="1">
-      <c r="A3" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="C3" s="29" t="s">
-        <v>135</v>
-      </c>
-      <c r="D3" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="E3" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="H3" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="I3" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="J3" s="16"/>
-      <c r="K3" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="L3" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="M3" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="N3" s="18">
-        <v>26393</v>
-      </c>
-      <c r="O3" s="19">
-        <v>46043</v>
-      </c>
-      <c r="P3" s="20"/>
-      <c r="Q3" s="21">
-        <v>1</v>
-      </c>
-      <c r="R3" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="S3" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="T3" s="16" t="s">
-        <v>132</v>
-      </c>
-      <c r="U3" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="V3" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="W3" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="X3" s="22">
-        <v>1</v>
-      </c>
-      <c r="Y3" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="Z3" s="24"/>
-      <c r="AA3" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="AB3" s="28">
-        <v>3501810</v>
-      </c>
-      <c r="AC3" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="AD3" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="AE3" s="19">
-        <v>46043</v>
-      </c>
-      <c r="AF3" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="AG3" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="AH3" s="19">
-        <v>46043</v>
-      </c>
-      <c r="AI3" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="AJ3" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="AK3" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="AL3" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="AM3" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="AN3" s="16"/>
-      <c r="AO3" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="AP3" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="AQ3" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="AR3" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="AS3" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="AT3" s="25">
-        <v>46171</v>
-      </c>
-      <c r="AU3" s="15">
-        <v>1</v>
-      </c>
-      <c r="AV3" s="15">
-        <v>1</v>
-      </c>
-      <c r="AW3" s="15">
-        <v>4</v>
-      </c>
-      <c r="AX3" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="AY3" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="AZ3" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="BA3" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="BB3" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="BC3" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="BD3" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="BE3" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="BF3" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="BG3" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="BH3" s="15">
-        <v>4801001</v>
-      </c>
-      <c r="BI3" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="BJ3" s="15">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1830,16 +1419,33 @@
   <conditionalFormatting sqref="C1:C1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
-  <hyperlinks>
-    <hyperlink ref="K3" r:id="rId1" xr:uid="{CD9B215C-075B-48B2-B03E-AC7FD645FC7C}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="dbcdebb2-cf80-47cd-9ce4-da05099ac60d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="01928591-29d3-40bf-897b-6c60acb0e16c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100D2281554FBC400488A53CD5E4CF21A4D" ma:contentTypeVersion="18" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="065bbd2080efe63d96717a72b278d73c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="dbcdebb2-cf80-47cd-9ce4-da05099ac60d" xmlns:ns3="cb6b3d82-e657-49dc-ab00-8f11ccd10803" xmlns:ns4="01928591-29d3-40bf-897b-6c60acb0e16c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8c7732d0698db1a95db4353621cbd5f0" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="dbcdebb2-cf80-47cd-9ce4-da05099ac60d"/>
@@ -2099,27 +1705,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{949287C3-ECA2-45B9-9545-B08D69B2FC27}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dbcdebb2-cf80-47cd-9ce4-da05099ac60d"/>
+    <ds:schemaRef ds:uri="01928591-29d3-40bf-897b-6c60acb0e16c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="dbcdebb2-cf80-47cd-9ce4-da05099ac60d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="01928591-29d3-40bf-897b-6c60acb0e16c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCF802FC-1CD7-42AF-A863-18B2CC423DDF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48D07738-D97B-46EB-A622-06D6123B5DFD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2137,23 +1742,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCF802FC-1CD7-42AF-A863-18B2CC423DDF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{949287C3-ECA2-45B9-9545-B08D69B2FC27}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dbcdebb2-cf80-47cd-9ce4-da05099ac60d"/>
-    <ds:schemaRef ds:uri="01928591-29d3-40bf-897b-6c60acb0e16c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>